<commit_message>
Initial commit: Cluenex blog
</commit_message>
<xml_diff>
--- a/Cluenex Content.xlsx
+++ b/Cluenex Content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Claude\Projects\Cluenex Content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2191DE8-16BE-4096-9FF9-F358925E3BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60BD60B-0852-4EF6-84A8-F3D0D0710FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98ACFBED-9EB7-4642-8712-CDA9C50EE277}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
   <si>
     <t>TECHNICAL ANALYSIS (Core evergreen, heavily searched)</t>
   </si>
@@ -364,14 +364,515 @@
   </si>
   <si>
     <t>100. How to use Cluenex to run a complete stock analysis in under 5 minutes — step-by-step walkthrough</t>
+  </si>
+  <si>
+    <t>cluenex.com/learn/</t>
+  </si>
+  <si>
+    <t>Long-form definitive guides. Each category gets a landing page + individual article pages.</t>
+  </si>
+  <si>
+    <r>
+      <t>Technical Analysis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/learn/technical-analysis/</t>
+    </r>
+  </si>
+  <si>
+    <t>/rsi-explained</t>
+  </si>
+  <si>
+    <t>/macd-explained</t>
+  </si>
+  <si>
+    <t>/moving-averages</t>
+  </si>
+  <si>
+    <t>/bollinger-bands</t>
+  </si>
+  <si>
+    <t>/candlestick-patterns</t>
+  </si>
+  <si>
+    <t>/support-resistance</t>
+  </si>
+  <si>
+    <t>/fibonacci-retracements</t>
+  </si>
+  <si>
+    <t>/volume-analysis</t>
+  </si>
+  <si>
+    <t>/trendlines</t>
+  </si>
+  <si>
+    <t>/breakout-vs-fakeout</t>
+  </si>
+  <si>
+    <t>/relative-strength</t>
+  </si>
+  <si>
+    <t>/vix-explained</t>
+  </si>
+  <si>
+    <r>
+      <t>Smart Money Concepts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/learn/smart-money/</t>
+    </r>
+  </si>
+  <si>
+    <t>/order-blocks</t>
+  </si>
+  <si>
+    <t>/fair-value-gaps</t>
+  </si>
+  <si>
+    <t>/liquidity-hunting</t>
+  </si>
+  <si>
+    <t>/supply-demand-zones</t>
+  </si>
+  <si>
+    <t>/market-structure</t>
+  </si>
+  <si>
+    <t>/choch-explained</t>
+  </si>
+  <si>
+    <t>/inducement-stop-hunts</t>
+  </si>
+  <si>
+    <t>/vwap-institutional-use</t>
+  </si>
+  <si>
+    <t>/opening-range-breakout</t>
+  </si>
+  <si>
+    <r>
+      <t>Fundamental Analysis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/learn/fundamental-analysis/</t>
+    </r>
+  </si>
+  <si>
+    <t>/how-to-read-earnings</t>
+  </si>
+  <si>
+    <t>/pe-ratio</t>
+  </si>
+  <si>
+    <t>/forward-vs-trailing-pe</t>
+  </si>
+  <si>
+    <t>/peg-ratio</t>
+  </si>
+  <si>
+    <t>/price-to-sales</t>
+  </si>
+  <si>
+    <t>/reading-balance-sheet</t>
+  </si>
+  <si>
+    <t>/free-cash-flow</t>
+  </si>
+  <si>
+    <t>/ebitda</t>
+  </si>
+  <si>
+    <t>/economic-moat</t>
+  </si>
+  <si>
+    <t>/profit-margins</t>
+  </si>
+  <si>
+    <t>/revenue-guidance</t>
+  </si>
+  <si>
+    <t>/debt-analysis</t>
+  </si>
+  <si>
+    <t>/insider-buying-selling</t>
+  </si>
+  <si>
+    <t>/short-interest</t>
+  </si>
+  <si>
+    <t>/stock-buybacks</t>
+  </si>
+  <si>
+    <r>
+      <t>Portfolio &amp; Risk Management</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/learn/portfolio-management/</t>
+    </r>
+  </si>
+  <si>
+    <t>/position-sizing</t>
+  </si>
+  <si>
+    <t>/stop-loss-methods</t>
+  </si>
+  <si>
+    <t>/risk-reward-ratio</t>
+  </si>
+  <si>
+    <t>/portfolio-diversification</t>
+  </si>
+  <si>
+    <t>/portfolio-beta</t>
+  </si>
+  <si>
+    <t>/cutting-losses-vs-holding</t>
+  </si>
+  <si>
+    <t>/dollar-cost-averaging</t>
+  </si>
+  <si>
+    <t>/tax-loss-harvesting</t>
+  </si>
+  <si>
+    <t>/hedging-with-etfs</t>
+  </si>
+  <si>
+    <t>/maximum-drawdown</t>
+  </si>
+  <si>
+    <r>
+      <t>Stock Screening &amp; Selection</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/learn/stock-screening/</t>
+    </r>
+  </si>
+  <si>
+    <t>/how-to-use-stock-screener</t>
+  </si>
+  <si>
+    <t>/momentum-investing</t>
+  </si>
+  <si>
+    <t>/finding-stocks-before-breakout</t>
+  </si>
+  <si>
+    <t>/sentiment-analysis</t>
+  </si>
+  <si>
+    <t>/earnings-countdown-strategy</t>
+  </si>
+  <si>
+    <t>/how-to-build-watchlist</t>
+  </si>
+  <si>
+    <t>/growth-vs-value-stocks</t>
+  </si>
+  <si>
+    <t>/relative-volume</t>
+  </si>
+  <si>
+    <t>/float-and-why-it-matters</t>
+  </si>
+  <si>
+    <t>cluenex.com/glossary/</t>
+  </si>
+  <si>
+    <t>Short, precise definitions. Each term is its own page with links to the full /learn/ guide.</t>
+  </si>
+  <si>
+    <t>Categories within glossary:</t>
+  </si>
+  <si>
+    <r>
+      <t>Technical Terms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — RSI, MACD, VWAP, ATR, EMA, SMA, Bollinger Bands, etc.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Fundamental Terms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — P/E, EPS, EBITDA, FCF, ROE, P/S, PEG, etc.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Options Terms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — IV, Delta, Gamma, Theta, Vega, OI, 0DTE, etc.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Market Terms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — Bull/Bear market, Circuit breaker, Short squeeze, Float, etc.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SMC Terms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — Order block, FVG, BOS, CHOCH, Inducement, etc.</t>
+    </r>
+  </si>
+  <si>
+    <t>cluenex.com/blog/</t>
+  </si>
+  <si>
+    <t>Timely, trend-driven content. Categories here are tags/filters, not subfolders.</t>
+  </si>
+  <si>
+    <t>Macro &amp; Market Analysis</t>
+  </si>
+  <si>
+    <t>Fed rate decision impacts</t>
+  </si>
+  <si>
+    <t>Tariff and trade war market effects</t>
+  </si>
+  <si>
+    <t>CPI/PCE reaction breakdowns</t>
+  </si>
+  <si>
+    <t>Yield curve analysis</t>
+  </si>
+  <si>
+    <t>Geopolitical event impact on markets</t>
+  </si>
+  <si>
+    <t>AI &amp; Technology Investing</t>
+  </si>
+  <si>
+    <t>AI stock valuation guides</t>
+  </si>
+  <si>
+    <t>Semiconductor cycle analysis</t>
+  </si>
+  <si>
+    <t>HALO stocks thesis</t>
+  </si>
+  <si>
+    <t>AI capex and infrastructure plays</t>
+  </si>
+  <si>
+    <t>Data center REITs</t>
+  </si>
+  <si>
+    <t>Market Themes</t>
+  </si>
+  <si>
+    <t>Sector rotation breakdowns</t>
+  </si>
+  <si>
+    <t>Magnificent Seven updates</t>
+  </si>
+  <si>
+    <t>Short squeeze candidates</t>
+  </si>
+  <si>
+    <t>IPO analysis</t>
+  </si>
+  <si>
+    <t>Earnings season previews/reviews</t>
+  </si>
+  <si>
+    <t>Cluenex Tutorials</t>
+  </si>
+  <si>
+    <t>How to run a full stock analysis on Cluenex</t>
+  </si>
+  <si>
+    <t>Using Cluenex sentiment scores</t>
+  </si>
+  <si>
+    <t>Reading Cluenex valuation badges</t>
+  </si>
+  <si>
+    <t>How to use the earnings countdown feature</t>
+  </si>
+  <si>
+    <t>Setting up your Cluenex watchlist</t>
+  </si>
+  <si>
+    <t>cluenex.com/compare/</t>
+  </si>
+  <si>
+    <t>Comparison pages are high-citation targets. LLMs frequently pull from "X vs Y" pages.</t>
+  </si>
+  <si>
+    <t>/compare/rsi-vs-macd</t>
+  </si>
+  <si>
+    <t>/compare/growth-vs-value-investing</t>
+  </si>
+  <si>
+    <t>/compare/etf-vs-individual-stocks</t>
+  </si>
+  <si>
+    <t>/compare/fundamental-vs-technical-analysis</t>
+  </si>
+  <si>
+    <t>/compare/cluenex-vs-finviz</t>
+  </si>
+  <si>
+    <t>/compare/cluenex-vs-tradingview</t>
+  </si>
+  <si>
+    <t>/compare/cluenex-vs-seeking-alpha</t>
+  </si>
+  <si>
+    <t>cluenex.com/methodology/</t>
+  </si>
+  <si>
+    <t>Single section, multiple pages. This is your authority anchor — explains how Cluenex produces its data.</t>
+  </si>
+  <si>
+    <t>/methodology/sentiment-scoring</t>
+  </si>
+  <si>
+    <t>/methodology/valuation-badges</t>
+  </si>
+  <si>
+    <t>/methodology/ai-insights</t>
+  </si>
+  <si>
+    <t>/methodology/earnings-data</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -385,6 +886,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -407,14 +913,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,585 +1243,1791 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F3ACC02-EC89-4232-85A1-7047B8DDC191}">
-  <dimension ref="B2:B143"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:U151"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:15" ht="18">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B4" s="2" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" spans="2:15">
+      <c r="B3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="2:15" ht="18">
+      <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B5" s="2" t="s">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="O4" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15">
+      <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="2:15">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="O6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15">
+      <c r="B7" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="2:15">
+      <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B9" s="2" t="s">
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="O8" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15">
+      <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B10" s="2" t="s">
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="2:15">
+      <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="O10" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15">
+      <c r="B11" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="O11" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15">
+      <c r="B12" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B13" s="2" t="s">
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="O12" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15">
+      <c r="B13" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B14" s="2" t="s">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="O13" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15">
+      <c r="B14" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B15" s="2" t="s">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="O14" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="O15" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15">
+      <c r="B16" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="2" t="s">
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="O16" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15">
+      <c r="B17" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="2" t="s">
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="O17" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15">
+      <c r="B18" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="O18" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="O19" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="O20" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="21" spans="2:15">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="O21" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15" ht="18">
       <c r="B22" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B24" s="2" t="s">
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="2:15">
+      <c r="B23" s="4"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="O23" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="24" spans="2:15">
+      <c r="B24" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B25" s="2" t="s">
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="O24" s="2"/>
+    </row>
+    <row r="25" spans="2:15">
+      <c r="B25" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B26" s="2" t="s">
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="O25" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15">
+      <c r="B26" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B27" s="2" t="s">
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="O26" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15">
+      <c r="B27" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B28" s="2" t="s">
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="O27" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="2:15">
+      <c r="B28" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B29" s="2" t="s">
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="O28" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15">
+      <c r="B29" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B30" s="2" t="s">
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="O29" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15">
+      <c r="B30" s="5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B31" s="2" t="s">
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="O30" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15">
+      <c r="B31" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B32" s="2" t="s">
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="O31" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="2:15">
+      <c r="B32" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="2" t="s">
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="O32" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="2:15">
+      <c r="B33" s="5" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="37" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="O33" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="34" spans="2:15">
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" spans="2:15">
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="O35" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="2:15">
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="O36" s="2"/>
+    </row>
+    <row r="37" spans="2:15" ht="18">
       <c r="B37" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B38" s="2"/>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B39" s="2" t="s">
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="O37" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15">
+      <c r="B38" s="4"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="O38" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="39" spans="2:15">
+      <c r="B39" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B40" s="2" t="s">
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="O39" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="40" spans="2:15">
+      <c r="B40" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B41" s="2" t="s">
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="O40" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41" spans="2:15">
+      <c r="B41" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B42" s="2" t="s">
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="O41" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="2:15">
+      <c r="B42" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B43" s="2" t="s">
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="O42" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43" spans="2:15">
+      <c r="B43" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B44" s="2" t="s">
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="O43" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="44" spans="2:15">
+      <c r="B44" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B45" s="2" t="s">
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="O44" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="45" spans="2:15">
+      <c r="B45" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B46" s="2" t="s">
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="O45" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="46" spans="2:15">
+      <c r="B46" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B47" s="2" t="s">
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="O46" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" spans="2:15">
+      <c r="B47" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B48" s="2" t="s">
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="O47" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="48" spans="2:15">
+      <c r="B48" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="52" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="O48" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="2:21">
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="O49" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="50" spans="2:21">
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="O50" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="U50" s="3"/>
+    </row>
+    <row r="51" spans="2:21">
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="O51" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="U51" s="2"/>
+    </row>
+    <row r="52" spans="2:21" ht="18">
       <c r="B52" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B53" s="2"/>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B54" s="2" t="s">
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="U52" s="2"/>
+    </row>
+    <row r="53" spans="2:21">
+      <c r="B53" s="4"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+      <c r="O53" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="U53" s="2"/>
+    </row>
+    <row r="54" spans="2:21">
+      <c r="B54" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B55" s="2" t="s">
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="O54" s="2"/>
+      <c r="U54" s="2"/>
+    </row>
+    <row r="55" spans="2:21">
+      <c r="B55" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B56" s="2" t="s">
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+      <c r="O55" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="U55" s="2"/>
+    </row>
+    <row r="56" spans="2:21">
+      <c r="B56" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B57" s="2" t="s">
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+      <c r="O56" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="U56" s="2"/>
+    </row>
+    <row r="57" spans="2:21">
+      <c r="B57" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B58" s="2" t="s">
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="O57" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="U57" s="2"/>
+    </row>
+    <row r="58" spans="2:21">
+      <c r="B58" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B59" s="2" t="s">
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="O58" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="U58" s="2"/>
+    </row>
+    <row r="59" spans="2:21">
+      <c r="B59" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B60" s="2" t="s">
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+      <c r="O59" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="U59" s="2"/>
+    </row>
+    <row r="60" spans="2:21">
+      <c r="B60" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B61" s="2" t="s">
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="O60" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="U60" s="2"/>
+    </row>
+    <row r="61" spans="2:21">
+      <c r="B61" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B62" s="2" t="s">
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+      <c r="O61" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="62" spans="2:21">
+      <c r="B62" s="5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B63" s="2" t="s">
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+      <c r="O62" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="63" spans="2:21">
+      <c r="B63" s="5" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B64" s="2" t="s">
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+      <c r="O63" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="64" spans="2:21">
+      <c r="B64" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B65" s="2" t="s">
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="O64" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="65" spans="2:15">
+      <c r="B65" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B66" s="2" t="s">
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+    </row>
+    <row r="66" spans="2:15">
+      <c r="B66" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B67" s="2" t="s">
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+      <c r="O66" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="67" spans="2:15">
+      <c r="B67" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B68" s="2" t="s">
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+      <c r="O67" s="2"/>
+    </row>
+    <row r="68" spans="2:15">
+      <c r="B68" s="5" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="72" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+      <c r="O68" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="69" spans="2:15">
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+      <c r="O69" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="70" spans="2:15">
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="O70" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="71" spans="2:15">
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+      <c r="O71" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="72" spans="2:15" ht="18">
       <c r="B72" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B73" s="2"/>
-    </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B74" s="2" t="s">
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+      <c r="O72" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="73" spans="2:15">
+      <c r="B73" s="4"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+      <c r="O73" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="74" spans="2:15">
+      <c r="B74" s="5" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B75" s="2" t="s">
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="O74" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="75" spans="2:15">
+      <c r="B75" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B76" s="2" t="s">
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="O75" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="76" spans="2:15">
+      <c r="B76" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B77" s="2" t="s">
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="O76" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="77" spans="2:15">
+      <c r="B77" s="5" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B78" s="2" t="s">
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="3"/>
+      <c r="J77" s="3"/>
+    </row>
+    <row r="78" spans="2:15" ht="18">
+      <c r="B78" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B79" s="2" t="s">
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="O78" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="79" spans="2:15">
+      <c r="B79" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B80" s="2" t="s">
+      <c r="C79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+    </row>
+    <row r="80" spans="2:15">
+      <c r="B80" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B81" s="2" t="s">
+      <c r="C80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+      <c r="O80" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="81" spans="2:15">
+      <c r="B81" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B82" s="2" t="s">
+      <c r="C81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+    </row>
+    <row r="82" spans="2:15">
+      <c r="B82" s="5" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B83" s="2" t="s">
+      <c r="C82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="3"/>
+      <c r="J82" s="3"/>
+      <c r="O82" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="83" spans="2:15">
+      <c r="B83" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="87" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3"/>
+      <c r="J83" s="3"/>
+      <c r="O83" s="2"/>
+    </row>
+    <row r="84" spans="2:15">
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="3"/>
+      <c r="J84" s="3"/>
+      <c r="O84" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="85" spans="2:15">
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+      <c r="O85" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="86" spans="2:15">
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="3"/>
+      <c r="J86" s="3"/>
+      <c r="O86" s="4" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="87" spans="2:15" ht="18">
       <c r="B87" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B88" s="2"/>
-    </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B89" s="2" t="s">
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+      <c r="O87" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="88" spans="2:15">
+      <c r="B88" s="4"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
+      <c r="I88" s="3"/>
+      <c r="J88" s="3"/>
+      <c r="O88" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="89" spans="2:15">
+      <c r="B89" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B90" s="2" t="s">
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="3"/>
+      <c r="J89" s="3"/>
+    </row>
+    <row r="90" spans="2:15">
+      <c r="B90" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B91" s="2" t="s">
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+    </row>
+    <row r="91" spans="2:15">
+      <c r="B91" s="5" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B92" s="2" t="s">
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+      <c r="I91" s="3"/>
+      <c r="J91" s="3"/>
+    </row>
+    <row r="92" spans="2:15" ht="18">
+      <c r="B92" s="5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B93" s="2" t="s">
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3"/>
+      <c r="J92" s="3"/>
+      <c r="O92" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="93" spans="2:15">
+      <c r="B93" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B94" s="2" t="s">
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+      <c r="I93" s="3"/>
+      <c r="J93" s="3"/>
+    </row>
+    <row r="94" spans="2:15">
+      <c r="B94" s="5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B95" s="2" t="s">
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+      <c r="I94" s="3"/>
+      <c r="J94" s="3"/>
+      <c r="O94" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="95" spans="2:15">
+      <c r="B95" s="5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B96" s="2" t="s">
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3"/>
+      <c r="J95" s="3"/>
+    </row>
+    <row r="96" spans="2:15">
+      <c r="B96" s="5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B97" s="2" t="s">
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+      <c r="I96" s="3"/>
+      <c r="J96" s="3"/>
+      <c r="O96" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="97" spans="2:15">
+      <c r="B97" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B98" s="2" t="s">
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+      <c r="I97" s="3"/>
+      <c r="J97" s="3"/>
+      <c r="O97" s="2"/>
+    </row>
+    <row r="98" spans="2:15">
+      <c r="B98" s="5" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="102" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3"/>
+      <c r="J98" s="3"/>
+      <c r="O98" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="99" spans="2:15">
+      <c r="O99" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="100" spans="2:15">
+      <c r="O100" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="101" spans="2:15">
+      <c r="O101" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="102" spans="2:15" ht="18">
       <c r="B102" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O102" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="103" spans="2:15">
       <c r="B103" s="2"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:15">
       <c r="B104" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O104" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="105" spans="2:15">
       <c r="B105" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O105" s="2"/>
+    </row>
+    <row r="106" spans="2:15">
       <c r="B106" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O106" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="107" spans="2:15">
       <c r="B107" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O107" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="108" spans="2:15">
       <c r="B108" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O108" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="109" spans="2:15">
       <c r="B109" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O109" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="110" spans="2:15">
       <c r="B110" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O110" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="111" spans="2:15">
       <c r="B111" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:15">
       <c r="B112" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O112" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="113" spans="2:15">
       <c r="B113" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="117" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+      <c r="O113" s="2"/>
+    </row>
+    <row r="114" spans="2:15">
+      <c r="O114" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="115" spans="2:15">
+      <c r="O115" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="116" spans="2:15">
+      <c r="O116" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="117" spans="2:15" ht="18">
       <c r="B117" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O117" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="118" spans="2:15">
       <c r="B118" s="2"/>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O118" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="119" spans="2:15">
       <c r="B119" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:15">
       <c r="B120" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O120" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="121" spans="2:15">
       <c r="B121" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O121" s="2"/>
+    </row>
+    <row r="122" spans="2:15">
       <c r="B122" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O122" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="123" spans="2:15">
       <c r="B123" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O123" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="124" spans="2:15">
       <c r="B124" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O124" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="125" spans="2:15">
       <c r="B125" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O125" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="126" spans="2:15">
       <c r="B126" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O126" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="127" spans="2:15">
       <c r="B127" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:15">
       <c r="B128" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="132" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:15" ht="18">
+      <c r="O130" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="132" spans="2:15" ht="18">
       <c r="B132" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O132" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="133" spans="2:15">
       <c r="B133" s="2"/>
-    </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O133" s="2"/>
+    </row>
+    <row r="134" spans="2:15">
       <c r="B134" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O134" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="135" spans="2:15">
       <c r="B135" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O135" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="136" spans="2:15">
       <c r="B136" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O136" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="137" spans="2:15">
       <c r="B137" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O137" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="138" spans="2:15">
       <c r="B138" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O138" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="139" spans="2:15">
       <c r="B139" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O139" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="140" spans="2:15">
       <c r="B140" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="O140" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="141" spans="2:15">
       <c r="B141" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:15">
       <c r="B142" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:15">
       <c r="B143" s="2" t="s">
         <v>108</v>
       </c>
     </row>
+    <row r="144" spans="2:15" ht="18">
+      <c r="O144" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="146" spans="15:15">
+      <c r="O146" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="147" spans="15:15">
+      <c r="O147" s="2"/>
+    </row>
+    <row r="148" spans="15:15">
+      <c r="O148" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="149" spans="15:15">
+      <c r="O149" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="150" spans="15:15">
+      <c r="O150" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="151" spans="15:15">
+      <c r="O151" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>